<commit_message>
📊 Update NAIC content history - 2025-08-02
</commit_message>
<xml_diff>
--- a/docs/content_history/pbr-2025-vm20-table-f-g-current-spreads.xlsx
+++ b/docs/content_history/pbr-2025-vm20-table-f-g-current-spreads.xlsx
@@ -1,25 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28925"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\PBR\VM20_VM22_ProductSupport\PBR Production Web Data\Current Year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E49C4DE-3C52-4585-B5C8-D2E8FD158614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84C6373A-1A56-4ED1-8093-6C1597467A51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="795" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" tabRatio="795" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="June_2025" sheetId="17" r:id="rId1"/>
-    <sheet name="May_2025" sheetId="16" r:id="rId2"/>
-    <sheet name="April_2025" sheetId="15" r:id="rId3"/>
-    <sheet name="March_2025" sheetId="14" r:id="rId4"/>
-    <sheet name="February_2025" sheetId="13" r:id="rId5"/>
-    <sheet name="January_2025" sheetId="12" r:id="rId6"/>
-    <sheet name="LEGAL DISCLAIMER" sheetId="11" r:id="rId7"/>
+    <sheet name="July_2025" sheetId="18" r:id="rId1"/>
+    <sheet name="June_2025" sheetId="17" r:id="rId2"/>
+    <sheet name="May_2025" sheetId="16" r:id="rId3"/>
+    <sheet name="April_2025" sheetId="15" r:id="rId4"/>
+    <sheet name="March_2025" sheetId="14" r:id="rId5"/>
+    <sheet name="February_2025" sheetId="13" r:id="rId6"/>
+    <sheet name="January_2025" sheetId="12" r:id="rId7"/>
+    <sheet name="LEGAL DISCLAIMER" sheetId="11" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="40">
   <si>
     <t>Table F (01/31/2025)  Investment Grade Current Benchmark Spreads (in bps)</t>
   </si>
@@ -150,6 +151,12 @@
   </si>
   <si>
     <t>Table G. (06/30/2025) Below Investment Grade Current Benchmark Spreads (in bps)</t>
+  </si>
+  <si>
+    <t>Table F (07/31/2025)  Investment Grade Current Benchmark Spreads (in bps)</t>
+  </si>
+  <si>
+    <t>Table G. (07/31/2025) Below Investment Grade Current Benchmark Spreads (in bps)</t>
   </si>
 </sst>
 </file>
@@ -415,7 +422,7 @@
                   <a14:compatExt spid="_x0000_s4104"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-000008100000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0600-000008100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -736,15 +743,2338 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51E35BE4-EF70-41CF-AF12-CCB5BAE8DA8A}">
+  <dimension ref="A1:W35"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="11.08984375" customWidth="1"/>
+    <col min="13" max="23" width="11.08984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="M1" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="N1" s="13"/>
+      <c r="O1" s="13"/>
+      <c r="P1" s="13"/>
+      <c r="Q1" s="13"/>
+      <c r="R1" s="13"/>
+      <c r="S1" s="13"/>
+      <c r="T1" s="13"/>
+      <c r="U1" s="13"/>
+      <c r="V1" s="13"/>
+      <c r="W1" s="14"/>
+    </row>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="11"/>
+      <c r="J2" s="11"/>
+      <c r="K2" s="11"/>
+      <c r="M2" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="N2" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="O2" s="11"/>
+      <c r="P2" s="11"/>
+      <c r="Q2" s="11"/>
+      <c r="R2" s="11"/>
+      <c r="S2" s="11"/>
+      <c r="T2" s="11"/>
+      <c r="U2" s="11"/>
+      <c r="V2" s="11"/>
+      <c r="W2" s="11"/>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A3" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="5">
+        <v>1</v>
+      </c>
+      <c r="C3" s="5">
+        <v>2</v>
+      </c>
+      <c r="D3" s="5">
+        <v>3</v>
+      </c>
+      <c r="E3" s="5">
+        <v>4</v>
+      </c>
+      <c r="F3" s="5">
+        <v>5</v>
+      </c>
+      <c r="G3" s="5">
+        <v>6</v>
+      </c>
+      <c r="H3" s="5">
+        <v>7</v>
+      </c>
+      <c r="I3" s="5">
+        <v>8</v>
+      </c>
+      <c r="J3" s="5">
+        <v>9</v>
+      </c>
+      <c r="K3" s="5">
+        <v>10</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="N3" s="5">
+        <v>11</v>
+      </c>
+      <c r="O3" s="5">
+        <v>12</v>
+      </c>
+      <c r="P3" s="5">
+        <v>13</v>
+      </c>
+      <c r="Q3" s="5">
+        <v>14</v>
+      </c>
+      <c r="R3" s="5">
+        <v>15</v>
+      </c>
+      <c r="S3" s="5">
+        <v>16</v>
+      </c>
+      <c r="T3" s="5">
+        <v>17</v>
+      </c>
+      <c r="U3" s="5">
+        <v>18</v>
+      </c>
+      <c r="V3" s="5">
+        <v>19</v>
+      </c>
+      <c r="W3" s="5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="M4" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="T4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="U4" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="W4" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A5" s="5">
+        <v>1</v>
+      </c>
+      <c r="B5" s="8">
+        <v>0.31</v>
+      </c>
+      <c r="C5" s="8">
+        <v>10.38</v>
+      </c>
+      <c r="D5" s="8">
+        <v>20.440000000000001</v>
+      </c>
+      <c r="E5" s="8">
+        <v>26.83</v>
+      </c>
+      <c r="F5" s="8">
+        <v>33.22</v>
+      </c>
+      <c r="G5" s="8">
+        <v>39.61</v>
+      </c>
+      <c r="H5" s="8">
+        <v>46.2</v>
+      </c>
+      <c r="I5" s="8">
+        <v>52.78</v>
+      </c>
+      <c r="J5" s="8">
+        <v>59.36</v>
+      </c>
+      <c r="K5" s="8">
+        <v>101.84</v>
+      </c>
+      <c r="M5" s="9">
+        <v>1</v>
+      </c>
+      <c r="N5" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O5" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P5" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q5" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R5" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S5" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T5" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U5" s="8">
+        <v>824</v>
+      </c>
+      <c r="V5" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W5" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A6" s="5">
+        <v>2</v>
+      </c>
+      <c r="B6" s="8">
+        <v>8.27</v>
+      </c>
+      <c r="C6" s="8">
+        <v>17.04</v>
+      </c>
+      <c r="D6" s="8">
+        <v>25.8</v>
+      </c>
+      <c r="E6" s="8">
+        <v>32.369999999999997</v>
+      </c>
+      <c r="F6" s="8">
+        <v>38.93</v>
+      </c>
+      <c r="G6" s="8">
+        <v>45.5</v>
+      </c>
+      <c r="H6" s="8">
+        <v>53.29</v>
+      </c>
+      <c r="I6" s="8">
+        <v>61.08</v>
+      </c>
+      <c r="J6" s="8">
+        <v>68.87</v>
+      </c>
+      <c r="K6" s="8">
+        <v>106.6</v>
+      </c>
+      <c r="M6" s="9">
+        <v>2</v>
+      </c>
+      <c r="N6" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O6" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P6" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q6" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R6" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S6" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T6" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U6" s="8">
+        <v>824</v>
+      </c>
+      <c r="V6" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W6" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A7" s="5">
+        <v>3</v>
+      </c>
+      <c r="B7" s="8">
+        <v>16.23</v>
+      </c>
+      <c r="C7" s="8">
+        <v>23.7</v>
+      </c>
+      <c r="D7" s="8">
+        <v>31.16</v>
+      </c>
+      <c r="E7" s="8">
+        <v>37.9</v>
+      </c>
+      <c r="F7" s="8">
+        <v>44.65</v>
+      </c>
+      <c r="G7" s="8">
+        <v>51.39</v>
+      </c>
+      <c r="H7" s="8">
+        <v>60.39</v>
+      </c>
+      <c r="I7" s="8">
+        <v>69.38</v>
+      </c>
+      <c r="J7" s="8">
+        <v>78.37</v>
+      </c>
+      <c r="K7" s="8">
+        <v>111.35</v>
+      </c>
+      <c r="M7" s="9">
+        <v>3</v>
+      </c>
+      <c r="N7" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O7" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P7" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q7" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R7" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S7" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T7" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U7" s="8">
+        <v>824</v>
+      </c>
+      <c r="V7" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W7" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A8" s="5">
+        <v>4</v>
+      </c>
+      <c r="B8" s="8">
+        <v>24.19</v>
+      </c>
+      <c r="C8" s="8">
+        <v>30.36</v>
+      </c>
+      <c r="D8" s="8">
+        <v>36.520000000000003</v>
+      </c>
+      <c r="E8" s="8">
+        <v>43.44</v>
+      </c>
+      <c r="F8" s="8">
+        <v>50.36</v>
+      </c>
+      <c r="G8" s="8">
+        <v>57.28</v>
+      </c>
+      <c r="H8" s="8">
+        <v>67.48</v>
+      </c>
+      <c r="I8" s="8">
+        <v>77.680000000000007</v>
+      </c>
+      <c r="J8" s="8">
+        <v>87.88</v>
+      </c>
+      <c r="K8" s="8">
+        <v>116.1</v>
+      </c>
+      <c r="M8" s="9">
+        <v>4</v>
+      </c>
+      <c r="N8" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O8" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P8" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q8" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R8" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S8" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T8" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U8" s="8">
+        <v>824</v>
+      </c>
+      <c r="V8" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W8" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A9" s="5">
+        <v>5</v>
+      </c>
+      <c r="B9" s="8">
+        <v>26.29</v>
+      </c>
+      <c r="C9" s="8">
+        <v>32.380000000000003</v>
+      </c>
+      <c r="D9" s="8">
+        <v>38.47</v>
+      </c>
+      <c r="E9" s="8">
+        <v>46.57</v>
+      </c>
+      <c r="F9" s="8">
+        <v>54.68</v>
+      </c>
+      <c r="G9" s="8">
+        <v>62.78</v>
+      </c>
+      <c r="H9" s="8">
+        <v>73.19</v>
+      </c>
+      <c r="I9" s="8">
+        <v>83.59</v>
+      </c>
+      <c r="J9" s="8">
+        <v>94</v>
+      </c>
+      <c r="K9" s="8">
+        <v>119.16</v>
+      </c>
+      <c r="M9" s="9">
+        <v>5</v>
+      </c>
+      <c r="N9" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O9" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P9" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q9" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R9" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S9" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T9" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U9" s="8">
+        <v>824</v>
+      </c>
+      <c r="V9" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W9" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A10" s="5">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8">
+        <v>28.39</v>
+      </c>
+      <c r="C10" s="8">
+        <v>34.4</v>
+      </c>
+      <c r="D10" s="8">
+        <v>40.409999999999997</v>
+      </c>
+      <c r="E10" s="8">
+        <v>49.7</v>
+      </c>
+      <c r="F10" s="8">
+        <v>58.99</v>
+      </c>
+      <c r="G10" s="8">
+        <v>68.28</v>
+      </c>
+      <c r="H10" s="8">
+        <v>78.89</v>
+      </c>
+      <c r="I10" s="8">
+        <v>89.5</v>
+      </c>
+      <c r="J10" s="8">
+        <v>100.11</v>
+      </c>
+      <c r="K10" s="8">
+        <v>122.22</v>
+      </c>
+      <c r="M10" s="9">
+        <v>6</v>
+      </c>
+      <c r="N10" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O10" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P10" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q10" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R10" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S10" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T10" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U10" s="8">
+        <v>824</v>
+      </c>
+      <c r="V10" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W10" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A11" s="5">
+        <v>7</v>
+      </c>
+      <c r="B11" s="8">
+        <v>26.35</v>
+      </c>
+      <c r="C11" s="8">
+        <v>35.17</v>
+      </c>
+      <c r="D11" s="8">
+        <v>43.98</v>
+      </c>
+      <c r="E11" s="8">
+        <v>53.15</v>
+      </c>
+      <c r="F11" s="8">
+        <v>62.33</v>
+      </c>
+      <c r="G11" s="8">
+        <v>71.510000000000005</v>
+      </c>
+      <c r="H11" s="8">
+        <v>82.07</v>
+      </c>
+      <c r="I11" s="8">
+        <v>92.63</v>
+      </c>
+      <c r="J11" s="8">
+        <v>103.2</v>
+      </c>
+      <c r="K11" s="8">
+        <v>123.76</v>
+      </c>
+      <c r="M11" s="9">
+        <v>7</v>
+      </c>
+      <c r="N11" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O11" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P11" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q11" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R11" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S11" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T11" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U11" s="8">
+        <v>824</v>
+      </c>
+      <c r="V11" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W11" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A12" s="5">
+        <v>8</v>
+      </c>
+      <c r="B12" s="8">
+        <v>24.32</v>
+      </c>
+      <c r="C12" s="8">
+        <v>35.93</v>
+      </c>
+      <c r="D12" s="8">
+        <v>47.54</v>
+      </c>
+      <c r="E12" s="8">
+        <v>56.6</v>
+      </c>
+      <c r="F12" s="8">
+        <v>65.66</v>
+      </c>
+      <c r="G12" s="8">
+        <v>74.73</v>
+      </c>
+      <c r="H12" s="8">
+        <v>85.24</v>
+      </c>
+      <c r="I12" s="8">
+        <v>95.76</v>
+      </c>
+      <c r="J12" s="8">
+        <v>106.28</v>
+      </c>
+      <c r="K12" s="8">
+        <v>125.3</v>
+      </c>
+      <c r="M12" s="9">
+        <v>8</v>
+      </c>
+      <c r="N12" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O12" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P12" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q12" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R12" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S12" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T12" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U12" s="8">
+        <v>824</v>
+      </c>
+      <c r="V12" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W12" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A13" s="5">
+        <v>9</v>
+      </c>
+      <c r="B13" s="8">
+        <v>22.29</v>
+      </c>
+      <c r="C13" s="8">
+        <v>36.69</v>
+      </c>
+      <c r="D13" s="8">
+        <v>51.1</v>
+      </c>
+      <c r="E13" s="8">
+        <v>60.05</v>
+      </c>
+      <c r="F13" s="8">
+        <v>69</v>
+      </c>
+      <c r="G13" s="8">
+        <v>77.95</v>
+      </c>
+      <c r="H13" s="8">
+        <v>88.42</v>
+      </c>
+      <c r="I13" s="8">
+        <v>98.89</v>
+      </c>
+      <c r="J13" s="8">
+        <v>109.36</v>
+      </c>
+      <c r="K13" s="8">
+        <v>126.84</v>
+      </c>
+      <c r="M13" s="9">
+        <v>9</v>
+      </c>
+      <c r="N13" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O13" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P13" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q13" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R13" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S13" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T13" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U13" s="8">
+        <v>824</v>
+      </c>
+      <c r="V13" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W13" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A14" s="5">
+        <v>10</v>
+      </c>
+      <c r="B14" s="8">
+        <v>23.4</v>
+      </c>
+      <c r="C14" s="8">
+        <v>37.64</v>
+      </c>
+      <c r="D14" s="8">
+        <v>51.88</v>
+      </c>
+      <c r="E14" s="8">
+        <v>60.64</v>
+      </c>
+      <c r="F14" s="8">
+        <v>69.400000000000006</v>
+      </c>
+      <c r="G14" s="8">
+        <v>78.16</v>
+      </c>
+      <c r="H14" s="8">
+        <v>88.85</v>
+      </c>
+      <c r="I14" s="8">
+        <v>99.54</v>
+      </c>
+      <c r="J14" s="8">
+        <v>110.22</v>
+      </c>
+      <c r="K14" s="8">
+        <v>127.28</v>
+      </c>
+      <c r="M14" s="9">
+        <v>10</v>
+      </c>
+      <c r="N14" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O14" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P14" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q14" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R14" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S14" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T14" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U14" s="8">
+        <v>824</v>
+      </c>
+      <c r="V14" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W14" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A15" s="5">
+        <v>11</v>
+      </c>
+      <c r="B15" s="8">
+        <v>24.52</v>
+      </c>
+      <c r="C15" s="8">
+        <v>38.590000000000003</v>
+      </c>
+      <c r="D15" s="8">
+        <v>52.66</v>
+      </c>
+      <c r="E15" s="8">
+        <v>61.23</v>
+      </c>
+      <c r="F15" s="8">
+        <v>69.8</v>
+      </c>
+      <c r="G15" s="8">
+        <v>78.37</v>
+      </c>
+      <c r="H15" s="8">
+        <v>89.27</v>
+      </c>
+      <c r="I15" s="8">
+        <v>100.18</v>
+      </c>
+      <c r="J15" s="8">
+        <v>111.08</v>
+      </c>
+      <c r="K15" s="8">
+        <v>127.71</v>
+      </c>
+      <c r="M15" s="9">
+        <v>11</v>
+      </c>
+      <c r="N15" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O15" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P15" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q15" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R15" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S15" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T15" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U15" s="8">
+        <v>824</v>
+      </c>
+      <c r="V15" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W15" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A16" s="5">
+        <v>12</v>
+      </c>
+      <c r="B16" s="8">
+        <v>25.64</v>
+      </c>
+      <c r="C16" s="8">
+        <v>39.54</v>
+      </c>
+      <c r="D16" s="8">
+        <v>53.44</v>
+      </c>
+      <c r="E16" s="8">
+        <v>61.82</v>
+      </c>
+      <c r="F16" s="8">
+        <v>70.2</v>
+      </c>
+      <c r="G16" s="8">
+        <v>78.58</v>
+      </c>
+      <c r="H16" s="8">
+        <v>89.7</v>
+      </c>
+      <c r="I16" s="8">
+        <v>100.82</v>
+      </c>
+      <c r="J16" s="8">
+        <v>111.95</v>
+      </c>
+      <c r="K16" s="8">
+        <v>128.13999999999999</v>
+      </c>
+      <c r="M16" s="9">
+        <v>12</v>
+      </c>
+      <c r="N16" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O16" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P16" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q16" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R16" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S16" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T16" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U16" s="8">
+        <v>824</v>
+      </c>
+      <c r="V16" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W16" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A17" s="5">
+        <v>13</v>
+      </c>
+      <c r="B17" s="8">
+        <v>26.76</v>
+      </c>
+      <c r="C17" s="8">
+        <v>40.49</v>
+      </c>
+      <c r="D17" s="8">
+        <v>54.22</v>
+      </c>
+      <c r="E17" s="8">
+        <v>62.41</v>
+      </c>
+      <c r="F17" s="8">
+        <v>70.599999999999994</v>
+      </c>
+      <c r="G17" s="8">
+        <v>78.790000000000006</v>
+      </c>
+      <c r="H17" s="8">
+        <v>90.13</v>
+      </c>
+      <c r="I17" s="8">
+        <v>101.47</v>
+      </c>
+      <c r="J17" s="8">
+        <v>112.81</v>
+      </c>
+      <c r="K17" s="8">
+        <v>128.57</v>
+      </c>
+      <c r="M17" s="9">
+        <v>13</v>
+      </c>
+      <c r="N17" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O17" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P17" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q17" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R17" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S17" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T17" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U17" s="8">
+        <v>824</v>
+      </c>
+      <c r="V17" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W17" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A18" s="5">
+        <v>14</v>
+      </c>
+      <c r="B18" s="8">
+        <v>27.88</v>
+      </c>
+      <c r="C18" s="8">
+        <v>41.44</v>
+      </c>
+      <c r="D18" s="8">
+        <v>55</v>
+      </c>
+      <c r="E18" s="8">
+        <v>63</v>
+      </c>
+      <c r="F18" s="8">
+        <v>71</v>
+      </c>
+      <c r="G18" s="8">
+        <v>79</v>
+      </c>
+      <c r="H18" s="8">
+        <v>90.55</v>
+      </c>
+      <c r="I18" s="8">
+        <v>102.11</v>
+      </c>
+      <c r="J18" s="8">
+        <v>113.67</v>
+      </c>
+      <c r="K18" s="8">
+        <v>129</v>
+      </c>
+      <c r="M18" s="9">
+        <v>14</v>
+      </c>
+      <c r="N18" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O18" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P18" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q18" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R18" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S18" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T18" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U18" s="8">
+        <v>824</v>
+      </c>
+      <c r="V18" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W18" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A19" s="5">
+        <v>15</v>
+      </c>
+      <c r="B19" s="8">
+        <v>29</v>
+      </c>
+      <c r="C19" s="8">
+        <v>42.39</v>
+      </c>
+      <c r="D19" s="8">
+        <v>55.78</v>
+      </c>
+      <c r="E19" s="8">
+        <v>63.59</v>
+      </c>
+      <c r="F19" s="8">
+        <v>71.400000000000006</v>
+      </c>
+      <c r="G19" s="8">
+        <v>79.2</v>
+      </c>
+      <c r="H19" s="8">
+        <v>90.98</v>
+      </c>
+      <c r="I19" s="8">
+        <v>102.75</v>
+      </c>
+      <c r="J19" s="8">
+        <v>114.53</v>
+      </c>
+      <c r="K19" s="8">
+        <v>129.43</v>
+      </c>
+      <c r="M19" s="9">
+        <v>15</v>
+      </c>
+      <c r="N19" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O19" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P19" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q19" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R19" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S19" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T19" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U19" s="8">
+        <v>824</v>
+      </c>
+      <c r="V19" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W19" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A20" s="5">
+        <v>16</v>
+      </c>
+      <c r="B20" s="8">
+        <v>30.12</v>
+      </c>
+      <c r="C20" s="8">
+        <v>43.34</v>
+      </c>
+      <c r="D20" s="8">
+        <v>56.56</v>
+      </c>
+      <c r="E20" s="8">
+        <v>64.180000000000007</v>
+      </c>
+      <c r="F20" s="8">
+        <v>71.8</v>
+      </c>
+      <c r="G20" s="8">
+        <v>79.41</v>
+      </c>
+      <c r="H20" s="8">
+        <v>91.4</v>
+      </c>
+      <c r="I20" s="8">
+        <v>103.4</v>
+      </c>
+      <c r="J20" s="8">
+        <v>115.39</v>
+      </c>
+      <c r="K20" s="8">
+        <v>129.86000000000001</v>
+      </c>
+      <c r="M20" s="9">
+        <v>16</v>
+      </c>
+      <c r="N20" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O20" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P20" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q20" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R20" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S20" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T20" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U20" s="8">
+        <v>824</v>
+      </c>
+      <c r="V20" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W20" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A21" s="5">
+        <v>17</v>
+      </c>
+      <c r="B21" s="8">
+        <v>31.24</v>
+      </c>
+      <c r="C21" s="8">
+        <v>44.29</v>
+      </c>
+      <c r="D21" s="8">
+        <v>57.34</v>
+      </c>
+      <c r="E21" s="8">
+        <v>64.77</v>
+      </c>
+      <c r="F21" s="8">
+        <v>72.19</v>
+      </c>
+      <c r="G21" s="8">
+        <v>79.62</v>
+      </c>
+      <c r="H21" s="8">
+        <v>91.83</v>
+      </c>
+      <c r="I21" s="8">
+        <v>104.04</v>
+      </c>
+      <c r="J21" s="8">
+        <v>116.25</v>
+      </c>
+      <c r="K21" s="8">
+        <v>130.29</v>
+      </c>
+      <c r="M21" s="9">
+        <v>17</v>
+      </c>
+      <c r="N21" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O21" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P21" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q21" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R21" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S21" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T21" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U21" s="8">
+        <v>824</v>
+      </c>
+      <c r="V21" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W21" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A22" s="5">
+        <v>18</v>
+      </c>
+      <c r="B22" s="8">
+        <v>32.35</v>
+      </c>
+      <c r="C22" s="8">
+        <v>45.24</v>
+      </c>
+      <c r="D22" s="8">
+        <v>58.12</v>
+      </c>
+      <c r="E22" s="8">
+        <v>65.36</v>
+      </c>
+      <c r="F22" s="8">
+        <v>72.59</v>
+      </c>
+      <c r="G22" s="8">
+        <v>79.83</v>
+      </c>
+      <c r="H22" s="8">
+        <v>92.26</v>
+      </c>
+      <c r="I22" s="8">
+        <v>104.68</v>
+      </c>
+      <c r="J22" s="8">
+        <v>117.11</v>
+      </c>
+      <c r="K22" s="8">
+        <v>130.72</v>
+      </c>
+      <c r="M22" s="9">
+        <v>18</v>
+      </c>
+      <c r="N22" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O22" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P22" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q22" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R22" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S22" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T22" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U22" s="8">
+        <v>824</v>
+      </c>
+      <c r="V22" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W22" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A23" s="5">
+        <v>19</v>
+      </c>
+      <c r="B23" s="8">
+        <v>33.47</v>
+      </c>
+      <c r="C23" s="8">
+        <v>46.19</v>
+      </c>
+      <c r="D23" s="8">
+        <v>58.9</v>
+      </c>
+      <c r="E23" s="8">
+        <v>65.95</v>
+      </c>
+      <c r="F23" s="8">
+        <v>72.989999999999995</v>
+      </c>
+      <c r="G23" s="8">
+        <v>80.040000000000006</v>
+      </c>
+      <c r="H23" s="8">
+        <v>92.68</v>
+      </c>
+      <c r="I23" s="8">
+        <v>105.33</v>
+      </c>
+      <c r="J23" s="8">
+        <v>117.97</v>
+      </c>
+      <c r="K23" s="8">
+        <v>131.15</v>
+      </c>
+      <c r="M23" s="9">
+        <v>19</v>
+      </c>
+      <c r="N23" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O23" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P23" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q23" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R23" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S23" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T23" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U23" s="8">
+        <v>824</v>
+      </c>
+      <c r="V23" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W23" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A24" s="5">
+        <v>20</v>
+      </c>
+      <c r="B24" s="8">
+        <v>34.590000000000003</v>
+      </c>
+      <c r="C24" s="8">
+        <v>47.14</v>
+      </c>
+      <c r="D24" s="8">
+        <v>59.68</v>
+      </c>
+      <c r="E24" s="8">
+        <v>66.540000000000006</v>
+      </c>
+      <c r="F24" s="8">
+        <v>73.39</v>
+      </c>
+      <c r="G24" s="8">
+        <v>80.25</v>
+      </c>
+      <c r="H24" s="8">
+        <v>93.11</v>
+      </c>
+      <c r="I24" s="8">
+        <v>105.97</v>
+      </c>
+      <c r="J24" s="8">
+        <v>118.83</v>
+      </c>
+      <c r="K24" s="8">
+        <v>131.58000000000001</v>
+      </c>
+      <c r="M24" s="9">
+        <v>20</v>
+      </c>
+      <c r="N24" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O24" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P24" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q24" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R24" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S24" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T24" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U24" s="8">
+        <v>824</v>
+      </c>
+      <c r="V24" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W24" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A25" s="5">
+        <v>21</v>
+      </c>
+      <c r="B25" s="8">
+        <v>35.71</v>
+      </c>
+      <c r="C25" s="8">
+        <v>48.09</v>
+      </c>
+      <c r="D25" s="8">
+        <v>60.46</v>
+      </c>
+      <c r="E25" s="8">
+        <v>67.13</v>
+      </c>
+      <c r="F25" s="8">
+        <v>73.790000000000006</v>
+      </c>
+      <c r="G25" s="8">
+        <v>80.459999999999994</v>
+      </c>
+      <c r="H25" s="8">
+        <v>93.54</v>
+      </c>
+      <c r="I25" s="8">
+        <v>106.61</v>
+      </c>
+      <c r="J25" s="8">
+        <v>119.69</v>
+      </c>
+      <c r="K25" s="8">
+        <v>132.01</v>
+      </c>
+      <c r="M25" s="9">
+        <v>21</v>
+      </c>
+      <c r="N25" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O25" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P25" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q25" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R25" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S25" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T25" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U25" s="8">
+        <v>824</v>
+      </c>
+      <c r="V25" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W25" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A26" s="5">
+        <v>22</v>
+      </c>
+      <c r="B26" s="8">
+        <v>36.83</v>
+      </c>
+      <c r="C26" s="8">
+        <v>49.03</v>
+      </c>
+      <c r="D26" s="8">
+        <v>61.24</v>
+      </c>
+      <c r="E26" s="8">
+        <v>67.72</v>
+      </c>
+      <c r="F26" s="8">
+        <v>74.19</v>
+      </c>
+      <c r="G26" s="8">
+        <v>80.67</v>
+      </c>
+      <c r="H26" s="8">
+        <v>93.96</v>
+      </c>
+      <c r="I26" s="8">
+        <v>107.26</v>
+      </c>
+      <c r="J26" s="8">
+        <v>120.55</v>
+      </c>
+      <c r="K26" s="8">
+        <v>132.44</v>
+      </c>
+      <c r="M26" s="9">
+        <v>22</v>
+      </c>
+      <c r="N26" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O26" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P26" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q26" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R26" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S26" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T26" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U26" s="8">
+        <v>824</v>
+      </c>
+      <c r="V26" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W26" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A27" s="5">
+        <v>23</v>
+      </c>
+      <c r="B27" s="8">
+        <v>37.950000000000003</v>
+      </c>
+      <c r="C27" s="8">
+        <v>49.98</v>
+      </c>
+      <c r="D27" s="8">
+        <v>62.02</v>
+      </c>
+      <c r="E27" s="8">
+        <v>68.31</v>
+      </c>
+      <c r="F27" s="8">
+        <v>74.59</v>
+      </c>
+      <c r="G27" s="8">
+        <v>80.88</v>
+      </c>
+      <c r="H27" s="8">
+        <v>94.39</v>
+      </c>
+      <c r="I27" s="8">
+        <v>107.9</v>
+      </c>
+      <c r="J27" s="8">
+        <v>121.41</v>
+      </c>
+      <c r="K27" s="8">
+        <v>132.87</v>
+      </c>
+      <c r="M27" s="9">
+        <v>23</v>
+      </c>
+      <c r="N27" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O27" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P27" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q27" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R27" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S27" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T27" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U27" s="8">
+        <v>824</v>
+      </c>
+      <c r="V27" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W27" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="28" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A28" s="5">
+        <v>24</v>
+      </c>
+      <c r="B28" s="8">
+        <v>39.07</v>
+      </c>
+      <c r="C28" s="8">
+        <v>50.93</v>
+      </c>
+      <c r="D28" s="8">
+        <v>62.8</v>
+      </c>
+      <c r="E28" s="8">
+        <v>68.900000000000006</v>
+      </c>
+      <c r="F28" s="8">
+        <v>74.989999999999995</v>
+      </c>
+      <c r="G28" s="8">
+        <v>81.09</v>
+      </c>
+      <c r="H28" s="8">
+        <v>94.82</v>
+      </c>
+      <c r="I28" s="8">
+        <v>108.54</v>
+      </c>
+      <c r="J28" s="8">
+        <v>122.27</v>
+      </c>
+      <c r="K28" s="8">
+        <v>133.30000000000001</v>
+      </c>
+      <c r="M28" s="9">
+        <v>24</v>
+      </c>
+      <c r="N28" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O28" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P28" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q28" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R28" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S28" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T28" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U28" s="8">
+        <v>824</v>
+      </c>
+      <c r="V28" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W28" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="29" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A29" s="5">
+        <v>25</v>
+      </c>
+      <c r="B29" s="8">
+        <v>40.19</v>
+      </c>
+      <c r="C29" s="8">
+        <v>51.88</v>
+      </c>
+      <c r="D29" s="8">
+        <v>63.58</v>
+      </c>
+      <c r="E29" s="8">
+        <v>69.48</v>
+      </c>
+      <c r="F29" s="8">
+        <v>75.39</v>
+      </c>
+      <c r="G29" s="8">
+        <v>81.3</v>
+      </c>
+      <c r="H29" s="8">
+        <v>95.24</v>
+      </c>
+      <c r="I29" s="8">
+        <v>109.19</v>
+      </c>
+      <c r="J29" s="8">
+        <v>123.13</v>
+      </c>
+      <c r="K29" s="8">
+        <v>133.72999999999999</v>
+      </c>
+      <c r="M29" s="9">
+        <v>25</v>
+      </c>
+      <c r="N29" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O29" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P29" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q29" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R29" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S29" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T29" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U29" s="8">
+        <v>824</v>
+      </c>
+      <c r="V29" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W29" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="30" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A30" s="5">
+        <v>26</v>
+      </c>
+      <c r="B30" s="8">
+        <v>41.31</v>
+      </c>
+      <c r="C30" s="8">
+        <v>52.83</v>
+      </c>
+      <c r="D30" s="8">
+        <v>64.36</v>
+      </c>
+      <c r="E30" s="8">
+        <v>70.069999999999993</v>
+      </c>
+      <c r="F30" s="8">
+        <v>75.790000000000006</v>
+      </c>
+      <c r="G30" s="8">
+        <v>81.5</v>
+      </c>
+      <c r="H30" s="8">
+        <v>95.67</v>
+      </c>
+      <c r="I30" s="8">
+        <v>109.83</v>
+      </c>
+      <c r="J30" s="8">
+        <v>123.99</v>
+      </c>
+      <c r="K30" s="8">
+        <v>134.16</v>
+      </c>
+      <c r="M30" s="9">
+        <v>26</v>
+      </c>
+      <c r="N30" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O30" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P30" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q30" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R30" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S30" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T30" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U30" s="8">
+        <v>824</v>
+      </c>
+      <c r="V30" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W30" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="31" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A31" s="5">
+        <v>27</v>
+      </c>
+      <c r="B31" s="8">
+        <v>42.42</v>
+      </c>
+      <c r="C31" s="8">
+        <v>53.78</v>
+      </c>
+      <c r="D31" s="8">
+        <v>65.14</v>
+      </c>
+      <c r="E31" s="8">
+        <v>70.66</v>
+      </c>
+      <c r="F31" s="8">
+        <v>76.19</v>
+      </c>
+      <c r="G31" s="8">
+        <v>81.709999999999994</v>
+      </c>
+      <c r="H31" s="8">
+        <v>96.09</v>
+      </c>
+      <c r="I31" s="8">
+        <v>110.47</v>
+      </c>
+      <c r="J31" s="8">
+        <v>124.86</v>
+      </c>
+      <c r="K31" s="8">
+        <v>134.59</v>
+      </c>
+      <c r="M31" s="9">
+        <v>27</v>
+      </c>
+      <c r="N31" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O31" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P31" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q31" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R31" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S31" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T31" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U31" s="8">
+        <v>824</v>
+      </c>
+      <c r="V31" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W31" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="32" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A32" s="5">
+        <v>28</v>
+      </c>
+      <c r="B32" s="8">
+        <v>43.54</v>
+      </c>
+      <c r="C32" s="8">
+        <v>54.73</v>
+      </c>
+      <c r="D32" s="8">
+        <v>65.92</v>
+      </c>
+      <c r="E32" s="8">
+        <v>71.25</v>
+      </c>
+      <c r="F32" s="8">
+        <v>76.59</v>
+      </c>
+      <c r="G32" s="8">
+        <v>81.92</v>
+      </c>
+      <c r="H32" s="8">
+        <v>96.52</v>
+      </c>
+      <c r="I32" s="8">
+        <v>111.12</v>
+      </c>
+      <c r="J32" s="8">
+        <v>125.72</v>
+      </c>
+      <c r="K32" s="8">
+        <v>135.02000000000001</v>
+      </c>
+      <c r="M32" s="9">
+        <v>28</v>
+      </c>
+      <c r="N32" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O32" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P32" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q32" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R32" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S32" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T32" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U32" s="8">
+        <v>824</v>
+      </c>
+      <c r="V32" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W32" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="33" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A33" s="5">
+        <v>29</v>
+      </c>
+      <c r="B33" s="8">
+        <v>44.66</v>
+      </c>
+      <c r="C33" s="8">
+        <v>55.68</v>
+      </c>
+      <c r="D33" s="8">
+        <v>66.7</v>
+      </c>
+      <c r="E33" s="8">
+        <v>71.84</v>
+      </c>
+      <c r="F33" s="8">
+        <v>76.989999999999995</v>
+      </c>
+      <c r="G33" s="8">
+        <v>82.13</v>
+      </c>
+      <c r="H33" s="8">
+        <v>96.95</v>
+      </c>
+      <c r="I33" s="8">
+        <v>111.76</v>
+      </c>
+      <c r="J33" s="8">
+        <v>126.58</v>
+      </c>
+      <c r="K33" s="8">
+        <v>135.44999999999999</v>
+      </c>
+      <c r="M33" s="9">
+        <v>29</v>
+      </c>
+      <c r="N33" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O33" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P33" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q33" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R33" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S33" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T33" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U33" s="8">
+        <v>824</v>
+      </c>
+      <c r="V33" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W33" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="34" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A34" s="5">
+        <v>30</v>
+      </c>
+      <c r="B34" s="8">
+        <v>45.78</v>
+      </c>
+      <c r="C34" s="8">
+        <v>56.63</v>
+      </c>
+      <c r="D34" s="8">
+        <v>67.48</v>
+      </c>
+      <c r="E34" s="8">
+        <v>72.430000000000007</v>
+      </c>
+      <c r="F34" s="8">
+        <v>77.39</v>
+      </c>
+      <c r="G34" s="8">
+        <v>82.34</v>
+      </c>
+      <c r="H34" s="8">
+        <v>97.37</v>
+      </c>
+      <c r="I34" s="8">
+        <v>112.41</v>
+      </c>
+      <c r="J34" s="8">
+        <v>127.44</v>
+      </c>
+      <c r="K34" s="8">
+        <v>135.88</v>
+      </c>
+      <c r="M34" s="9">
+        <v>30</v>
+      </c>
+      <c r="N34" s="8">
+        <v>144.33000000000001</v>
+      </c>
+      <c r="O34" s="8">
+        <v>189.08</v>
+      </c>
+      <c r="P34" s="8">
+        <v>233.84</v>
+      </c>
+      <c r="Q34" s="8">
+        <v>278.58999999999997</v>
+      </c>
+      <c r="R34" s="8">
+        <v>323.35000000000002</v>
+      </c>
+      <c r="S34" s="8">
+        <v>490.23</v>
+      </c>
+      <c r="T34" s="8">
+        <v>657.12</v>
+      </c>
+      <c r="U34" s="8">
+        <v>824</v>
+      </c>
+      <c r="V34" s="8">
+        <v>990.88</v>
+      </c>
+      <c r="W34" s="8">
+        <v>1157.77</v>
+      </c>
+    </row>
+    <row r="35" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A35" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B35" s="8">
+        <v>30.102333333333331</v>
+      </c>
+      <c r="C35" s="8">
+        <v>41.53</v>
+      </c>
+      <c r="D35" s="8">
+        <v>52.956666666666671</v>
+      </c>
+      <c r="E35" s="8">
+        <v>60.129666666666672</v>
+      </c>
+      <c r="F35" s="8">
+        <v>67.302666666666667</v>
+      </c>
+      <c r="G35" s="8">
+        <v>74.476000000000028</v>
+      </c>
+      <c r="H35" s="8">
+        <v>86.349333333333334</v>
+      </c>
+      <c r="I35" s="8">
+        <v>98.222333333333324</v>
+      </c>
+      <c r="J35" s="8">
+        <v>110.096</v>
+      </c>
+      <c r="K35" s="8">
+        <v>127.21166666666666</v>
+      </c>
+      <c r="M35" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="N35" s="10">
+        <v>144.32999999999996</v>
+      </c>
+      <c r="O35" s="10">
+        <v>189.07999999999996</v>
+      </c>
+      <c r="P35" s="10">
+        <v>233.84000000000009</v>
+      </c>
+      <c r="Q35" s="10">
+        <v>278.59000000000009</v>
+      </c>
+      <c r="R35" s="10">
+        <v>323.35000000000019</v>
+      </c>
+      <c r="S35" s="10">
+        <v>490.22999999999968</v>
+      </c>
+      <c r="T35" s="10">
+        <v>657.12000000000012</v>
+      </c>
+      <c r="U35" s="10">
+        <v>824</v>
+      </c>
+      <c r="V35" s="10">
+        <v>990.88000000000034</v>
+      </c>
+      <c r="W35" s="10">
+        <v>1157.7700000000002</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="M1:W1"/>
+    <mergeCell ref="N2:W2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9DB5B8B-0B3D-4D0C-9E6D-ACD327AE1B1B}">
   <dimension ref="A1:W35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.140625" customWidth="1"/>
-    <col min="13" max="23" width="11.140625" customWidth="1"/>
+    <col min="1" max="1" width="11.1796875" customWidth="1"/>
+    <col min="13" max="23" width="11.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>36</v>
       </c>
@@ -772,7 +3102,7 @@
       <c r="V1" s="13"/>
       <c r="W1" s="14"/>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -804,7 +3134,7 @@
       <c r="V2" s="11"/>
       <c r="W2" s="11"/>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
         <v>3</v>
       </c>
@@ -872,7 +3202,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>4</v>
       </c>
@@ -940,7 +3270,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
         <v>1</v>
       </c>
@@ -1008,7 +3338,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
         <v>2</v>
       </c>
@@ -1076,7 +3406,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
         <v>3</v>
       </c>
@@ -1144,7 +3474,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
         <v>4</v>
       </c>
@@ -1212,7 +3542,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
         <v>5</v>
       </c>
@@ -1280,7 +3610,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
         <v>6</v>
       </c>
@@ -1348,7 +3678,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
         <v>7</v>
       </c>
@@ -1416,7 +3746,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
         <v>8</v>
       </c>
@@ -1484,7 +3814,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
         <v>9</v>
       </c>
@@ -1552,7 +3882,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
         <v>10</v>
       </c>
@@ -1620,7 +3950,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
         <v>11</v>
       </c>
@@ -1688,7 +4018,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
         <v>12</v>
       </c>
@@ -1756,7 +4086,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
         <v>13</v>
       </c>
@@ -1824,7 +4154,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
         <v>14</v>
       </c>
@@ -1892,7 +4222,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
         <v>15</v>
       </c>
@@ -1960,7 +4290,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
         <v>16</v>
       </c>
@@ -2028,7 +4358,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
         <v>17</v>
       </c>
@@ -2096,7 +4426,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
         <v>18</v>
       </c>
@@ -2164,7 +4494,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
         <v>19</v>
       </c>
@@ -2232,7 +4562,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
         <v>20</v>
       </c>
@@ -2300,7 +4630,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
         <v>21</v>
       </c>
@@ -2368,7 +4698,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A26" s="5">
         <v>22</v>
       </c>
@@ -2436,7 +4766,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A27" s="5">
         <v>23</v>
       </c>
@@ -2504,7 +4834,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
         <v>24</v>
       </c>
@@ -2572,7 +4902,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A29" s="5">
         <v>25</v>
       </c>
@@ -2640,7 +4970,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A30" s="5">
         <v>26</v>
       </c>
@@ -2708,7 +5038,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A31" s="5">
         <v>27</v>
       </c>
@@ -2776,7 +5106,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
         <v>28</v>
       </c>
@@ -2844,7 +5174,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A33" s="5">
         <v>29</v>
       </c>
@@ -2912,7 +5242,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
         <v>30</v>
       </c>
@@ -2980,7 +5310,7 @@
         <v>1252.26</v>
       </c>
     </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
         <v>15</v>
       </c>
@@ -3058,16 +5388,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92FC35AE-E973-4CF9-9AE2-82A811E5E874}">
   <dimension ref="A1:W35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.140625" customWidth="1"/>
-    <col min="13" max="23" width="11.140625" customWidth="1"/>
+    <col min="1" max="1" width="11.1796875" customWidth="1"/>
+    <col min="13" max="23" width="11.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>34</v>
       </c>
@@ -3095,7 +5425,7 @@
       <c r="V1" s="13"/>
       <c r="W1" s="14"/>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -3127,7 +5457,7 @@
       <c r="V2" s="11"/>
       <c r="W2" s="11"/>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
         <v>3</v>
       </c>
@@ -3195,7 +5525,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>4</v>
       </c>
@@ -3263,7 +5593,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
         <v>1</v>
       </c>
@@ -3331,7 +5661,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
         <v>2</v>
       </c>
@@ -3399,7 +5729,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
         <v>3</v>
       </c>
@@ -3467,7 +5797,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
         <v>4</v>
       </c>
@@ -3535,7 +5865,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
         <v>5</v>
       </c>
@@ -3603,7 +5933,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
         <v>6</v>
       </c>
@@ -3671,7 +6001,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
         <v>7</v>
       </c>
@@ -3739,7 +6069,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
         <v>8</v>
       </c>
@@ -3807,7 +6137,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
         <v>9</v>
       </c>
@@ -3875,7 +6205,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
         <v>10</v>
       </c>
@@ -3943,7 +6273,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
         <v>11</v>
       </c>
@@ -4011,7 +6341,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
         <v>12</v>
       </c>
@@ -4079,7 +6409,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
         <v>13</v>
       </c>
@@ -4147,7 +6477,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
         <v>14</v>
       </c>
@@ -4215,7 +6545,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
         <v>15</v>
       </c>
@@ -4283,7 +6613,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
         <v>16</v>
       </c>
@@ -4351,7 +6681,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
         <v>17</v>
       </c>
@@ -4419,7 +6749,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
         <v>18</v>
       </c>
@@ -4487,7 +6817,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
         <v>19</v>
       </c>
@@ -4555,7 +6885,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
         <v>20</v>
       </c>
@@ -4623,7 +6953,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
         <v>21</v>
       </c>
@@ -4691,7 +7021,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A26" s="5">
         <v>22</v>
       </c>
@@ -4759,7 +7089,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A27" s="5">
         <v>23</v>
       </c>
@@ -4827,7 +7157,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
         <v>24</v>
       </c>
@@ -4895,7 +7225,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A29" s="5">
         <v>25</v>
       </c>
@@ -4963,7 +7293,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A30" s="5">
         <v>26</v>
       </c>
@@ -5031,7 +7361,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A31" s="5">
         <v>27</v>
       </c>
@@ -5099,7 +7429,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
         <v>28</v>
       </c>
@@ -5167,7 +7497,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A33" s="5">
         <v>29</v>
       </c>
@@ -5235,7 +7565,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
         <v>30</v>
       </c>
@@ -5303,7 +7633,7 @@
         <v>1244.73</v>
       </c>
     </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
         <v>15</v>
       </c>
@@ -5381,16 +7711,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAC8FFAC-4FD7-4739-8182-E5754BE58F0D}">
   <dimension ref="A1:W35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.140625" customWidth="1"/>
-    <col min="13" max="23" width="11.140625" customWidth="1"/>
+    <col min="1" max="1" width="11.1796875" customWidth="1"/>
+    <col min="13" max="23" width="11.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>32</v>
       </c>
@@ -5418,7 +7748,7 @@
       <c r="V1" s="13"/>
       <c r="W1" s="14"/>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -5450,7 +7780,7 @@
       <c r="V2" s="11"/>
       <c r="W2" s="11"/>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
         <v>3</v>
       </c>
@@ -5518,7 +7848,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>4</v>
       </c>
@@ -5586,7 +7916,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
         <v>1</v>
       </c>
@@ -5654,7 +7984,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
         <v>2</v>
       </c>
@@ -5722,7 +8052,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
         <v>3</v>
       </c>
@@ -5790,7 +8120,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
         <v>4</v>
       </c>
@@ -5858,7 +8188,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
         <v>5</v>
       </c>
@@ -5926,7 +8256,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
         <v>6</v>
       </c>
@@ -5994,7 +8324,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
         <v>7</v>
       </c>
@@ -6062,7 +8392,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
         <v>8</v>
       </c>
@@ -6130,7 +8460,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
         <v>9</v>
       </c>
@@ -6198,7 +8528,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
         <v>10</v>
       </c>
@@ -6266,7 +8596,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
         <v>11</v>
       </c>
@@ -6334,7 +8664,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
         <v>12</v>
       </c>
@@ -6402,7 +8732,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
         <v>13</v>
       </c>
@@ -6470,7 +8800,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
         <v>14</v>
       </c>
@@ -6538,7 +8868,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
         <v>15</v>
       </c>
@@ -6606,7 +8936,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
         <v>16</v>
       </c>
@@ -6674,7 +9004,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
         <v>17</v>
       </c>
@@ -6742,7 +9072,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
         <v>18</v>
       </c>
@@ -6810,7 +9140,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
         <v>19</v>
       </c>
@@ -6878,7 +9208,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
         <v>20</v>
       </c>
@@ -6946,7 +9276,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
         <v>21</v>
       </c>
@@ -7014,7 +9344,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A26" s="5">
         <v>22</v>
       </c>
@@ -7082,7 +9412,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A27" s="5">
         <v>23</v>
       </c>
@@ -7150,7 +9480,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
         <v>24</v>
       </c>
@@ -7218,7 +9548,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A29" s="5">
         <v>25</v>
       </c>
@@ -7286,7 +9616,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A30" s="5">
         <v>26</v>
       </c>
@@ -7354,7 +9684,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A31" s="5">
         <v>27</v>
       </c>
@@ -7422,7 +9752,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
         <v>28</v>
       </c>
@@ -7490,7 +9820,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A33" s="5">
         <v>29</v>
       </c>
@@ -7558,7 +9888,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
         <v>30</v>
       </c>
@@ -7626,7 +9956,7 @@
         <v>1374.27</v>
       </c>
     </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
         <v>15</v>
       </c>
@@ -7704,16 +10034,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{418E16CC-B113-45B8-9AB8-B4C2E0CD8BE4}">
   <dimension ref="A1:W35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.140625" customWidth="1"/>
-    <col min="13" max="23" width="11.140625" customWidth="1"/>
+    <col min="1" max="1" width="11.1796875" customWidth="1"/>
+    <col min="13" max="23" width="11.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>30</v>
       </c>
@@ -7741,7 +10071,7 @@
       <c r="V1" s="13"/>
       <c r="W1" s="14"/>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -7773,7 +10103,7 @@
       <c r="V2" s="11"/>
       <c r="W2" s="11"/>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
         <v>3</v>
       </c>
@@ -7841,7 +10171,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>4</v>
       </c>
@@ -7909,7 +10239,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
         <v>1</v>
       </c>
@@ -7977,7 +10307,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
         <v>2</v>
       </c>
@@ -8045,7 +10375,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
         <v>3</v>
       </c>
@@ -8113,7 +10443,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
         <v>4</v>
       </c>
@@ -8181,7 +10511,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
         <v>5</v>
       </c>
@@ -8249,7 +10579,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
         <v>6</v>
       </c>
@@ -8317,7 +10647,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
         <v>7</v>
       </c>
@@ -8385,7 +10715,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
         <v>8</v>
       </c>
@@ -8453,7 +10783,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
         <v>9</v>
       </c>
@@ -8521,7 +10851,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
         <v>10</v>
       </c>
@@ -8589,7 +10919,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
         <v>11</v>
       </c>
@@ -8657,7 +10987,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
         <v>12</v>
       </c>
@@ -8725,7 +11055,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
         <v>13</v>
       </c>
@@ -8793,7 +11123,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
         <v>14</v>
       </c>
@@ -8861,7 +11191,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
         <v>15</v>
       </c>
@@ -8929,7 +11259,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
         <v>16</v>
       </c>
@@ -8997,7 +11327,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
         <v>17</v>
       </c>
@@ -9065,7 +11395,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
         <v>18</v>
       </c>
@@ -9133,7 +11463,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
         <v>19</v>
       </c>
@@ -9201,7 +11531,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
         <v>20</v>
       </c>
@@ -9269,7 +11599,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
         <v>21</v>
       </c>
@@ -9337,7 +11667,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A26" s="5">
         <v>22</v>
       </c>
@@ -9405,7 +11735,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A27" s="5">
         <v>23</v>
       </c>
@@ -9473,7 +11803,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
         <v>24</v>
       </c>
@@ -9541,7 +11871,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A29" s="5">
         <v>25</v>
       </c>
@@ -9609,7 +11939,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A30" s="5">
         <v>26</v>
       </c>
@@ -9677,7 +12007,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A31" s="5">
         <v>27</v>
       </c>
@@ -9745,7 +12075,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
         <v>28</v>
       </c>
@@ -9813,7 +12143,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A33" s="5">
         <v>29</v>
       </c>
@@ -9881,7 +12211,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
         <v>30</v>
       </c>
@@ -9949,7 +12279,7 @@
         <v>1283.3499999999999</v>
       </c>
     </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
         <v>15</v>
       </c>
@@ -10027,16 +12357,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20021F30-9281-441A-B982-AE3628B68A09}">
   <dimension ref="A1:W35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.140625" customWidth="1"/>
-    <col min="13" max="23" width="11.140625" customWidth="1"/>
+    <col min="1" max="1" width="11.1796875" customWidth="1"/>
+    <col min="13" max="23" width="11.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>28</v>
       </c>
@@ -10064,7 +12394,7 @@
       <c r="V1" s="13"/>
       <c r="W1" s="14"/>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -10096,7 +12426,7 @@
       <c r="V2" s="11"/>
       <c r="W2" s="11"/>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
         <v>3</v>
       </c>
@@ -10164,7 +12494,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>4</v>
       </c>
@@ -10232,7 +12562,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
         <v>1</v>
       </c>
@@ -10300,7 +12630,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
         <v>2</v>
       </c>
@@ -10368,7 +12698,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
         <v>3</v>
       </c>
@@ -10436,7 +12766,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
         <v>4</v>
       </c>
@@ -10504,7 +12834,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
         <v>5</v>
       </c>
@@ -10572,7 +12902,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
         <v>6</v>
       </c>
@@ -10640,7 +12970,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
         <v>7</v>
       </c>
@@ -10708,7 +13038,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
         <v>8</v>
       </c>
@@ -10776,7 +13106,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
         <v>9</v>
       </c>
@@ -10844,7 +13174,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
         <v>10</v>
       </c>
@@ -10912,7 +13242,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
         <v>11</v>
       </c>
@@ -10980,7 +13310,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
         <v>12</v>
       </c>
@@ -11048,7 +13378,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
         <v>13</v>
       </c>
@@ -11116,7 +13446,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
         <v>14</v>
       </c>
@@ -11184,7 +13514,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
         <v>15</v>
       </c>
@@ -11252,7 +13582,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
         <v>16</v>
       </c>
@@ -11320,7 +13650,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
         <v>17</v>
       </c>
@@ -11388,7 +13718,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
         <v>18</v>
       </c>
@@ -11456,7 +13786,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
         <v>19</v>
       </c>
@@ -11524,7 +13854,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
         <v>20</v>
       </c>
@@ -11592,7 +13922,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
         <v>21</v>
       </c>
@@ -11660,7 +13990,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A26" s="5">
         <v>22</v>
       </c>
@@ -11728,7 +14058,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A27" s="5">
         <v>23</v>
       </c>
@@ -11796,7 +14126,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
         <v>24</v>
       </c>
@@ -11864,7 +14194,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A29" s="5">
         <v>25</v>
       </c>
@@ -11932,7 +14262,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A30" s="5">
         <v>26</v>
       </c>
@@ -12000,7 +14330,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A31" s="5">
         <v>27</v>
       </c>
@@ -12068,7 +14398,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
         <v>28</v>
       </c>
@@ -12136,7 +14466,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A33" s="5">
         <v>29</v>
       </c>
@@ -12204,7 +14534,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
         <v>30</v>
       </c>
@@ -12272,7 +14602,7 @@
         <v>1055.0899999999999</v>
       </c>
     </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
         <v>15</v>
       </c>
@@ -12350,16 +14680,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C329B72-B441-4A9C-B89A-4A1D58BE3ABB}">
   <dimension ref="A1:W35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.140625" customWidth="1"/>
-    <col min="13" max="23" width="11.140625" customWidth="1"/>
+    <col min="1" max="1" width="11.1796875" customWidth="1"/>
+    <col min="13" max="23" width="11.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -12387,7 +14717,7 @@
       <c r="V1" s="13"/>
       <c r="W1" s="14"/>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -12419,7 +14749,7 @@
       <c r="V2" s="11"/>
       <c r="W2" s="11"/>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
         <v>3</v>
       </c>
@@ -12487,7 +14817,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>4</v>
       </c>
@@ -12555,7 +14885,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
         <v>1</v>
       </c>
@@ -12623,7 +14953,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
         <v>2</v>
       </c>
@@ -12691,7 +15021,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
         <v>3</v>
       </c>
@@ -12759,7 +15089,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
         <v>4</v>
       </c>
@@ -12827,7 +15157,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
         <v>5</v>
       </c>
@@ -12895,7 +15225,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
         <v>6</v>
       </c>
@@ -12963,7 +15293,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
         <v>7</v>
       </c>
@@ -13031,7 +15361,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
         <v>8</v>
       </c>
@@ -13099,7 +15429,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
         <v>9</v>
       </c>
@@ -13167,7 +15497,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
         <v>10</v>
       </c>
@@ -13235,7 +15565,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
         <v>11</v>
       </c>
@@ -13303,7 +15633,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
         <v>12</v>
       </c>
@@ -13371,7 +15701,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
         <v>13</v>
       </c>
@@ -13439,7 +15769,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
         <v>14</v>
       </c>
@@ -13507,7 +15837,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
         <v>15</v>
       </c>
@@ -13575,7 +15905,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
         <v>16</v>
       </c>
@@ -13643,7 +15973,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
         <v>17</v>
       </c>
@@ -13711,7 +16041,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
         <v>18</v>
       </c>
@@ -13779,7 +16109,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
         <v>19</v>
       </c>
@@ -13847,7 +16177,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
         <v>20</v>
       </c>
@@ -13915,7 +16245,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
         <v>21</v>
       </c>
@@ -13983,7 +16313,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A26" s="5">
         <v>22</v>
       </c>
@@ -14051,7 +16381,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A27" s="5">
         <v>23</v>
       </c>
@@ -14119,7 +16449,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
         <v>24</v>
       </c>
@@ -14187,7 +16517,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A29" s="5">
         <v>25</v>
       </c>
@@ -14255,7 +16585,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A30" s="5">
         <v>26</v>
       </c>
@@ -14323,7 +16653,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A31" s="5">
         <v>27</v>
       </c>
@@ -14391,7 +16721,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
         <v>28</v>
       </c>
@@ -14459,7 +16789,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A33" s="5">
         <v>29</v>
       </c>
@@ -14527,7 +16857,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
         <v>30</v>
       </c>
@@ -14595,7 +16925,7 @@
         <v>968.77</v>
       </c>
     </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
         <v>15</v>
       </c>
@@ -14673,15 +17003,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <sheetPr codeName="Sheet9">
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="H31"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="31" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="8:8" x14ac:dyDescent="0.35">
       <c r="H31" s="1"/>
     </row>
   </sheetData>

</xml_diff>